<commit_message>
De Arima a Autoarima
</commit_message>
<xml_diff>
--- a/data/output/forecast_results.xlsx
+++ b/data/output/forecast_results.xlsx
@@ -472,17 +472,17 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3925.790035997552</v>
+        <v>3925.79003599756</v>
       </c>
       <c r="D2" t="n">
-        <v>4127.552351010443</v>
+        <v>4127.552351010448</v>
       </c>
       <c r="E2" t="n">
-        <v>25.56942245630023</v>
+        <v>25.56942245630032</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[20140.04304213168, 14303.797448665342, 11260.913084048872, 19622.90739303335, 9156.662006163253, 26757.10869901435, 21472.594346586764]</t>
+          <t>[20140.04304213169, 14303.797448665355, 11260.913084048887, 19622.90739303337, 9156.662006163273, 26757.108699014374, 21472.594346586793]</t>
         </is>
       </c>
     </row>
@@ -494,21 +494,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HW-add-add-a0.4-b0.8-g0.2</t>
+          <t>(5, 0, 3)</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>245.6394933808212</v>
+        <v>250.8257294371891</v>
       </c>
       <c r="D3" t="n">
-        <v>323.1724466626538</v>
+        <v>290.1722558268039</v>
       </c>
       <c r="E3" t="n">
-        <v>35.59639098586576</v>
+        <v>36.62604843082408</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[683.5802615395097, 1650.7047666218662, 934.2547110650983, 824.3802033438335, 712.6681985987466, 1146.0762799774807, 1082.0180275493872]</t>
+          <t>[734.7967849715267, 1291.1967353232162, 868.7311426137492, 1212.3203268543525, 1008.7444097226287, 915.7898888122093, 1211.2349421177785]</t>
         </is>
       </c>
     </row>
@@ -582,11 +582,11 @@
         <v>194.897187182262</v>
       </c>
       <c r="E6" t="n">
-        <v>51.35108673490244</v>
+        <v>51.35108673490243</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[845.6855874448174, 732.0919114289136, 436.82903591950924, 627.5750952457643, 327.0575831606717, 499.62943579598044, 697.8488015523835]</t>
+          <t>[845.6855874448173, 732.0919114289136, 436.8290359195093, 627.5750952457643, 327.0575831606717, 499.62943579598044, 697.8488015523835]</t>
         </is>
       </c>
     </row>
@@ -598,21 +598,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ARIMA(2,1,1)</t>
+          <t>(0, 1, 1)</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>820.327167512787</v>
+        <v>939.3338669463167</v>
       </c>
       <c r="D7" t="n">
-        <v>986.7932673726689</v>
+        <v>1067.359469846852</v>
       </c>
       <c r="E7" t="n">
-        <v>101.6145513947987</v>
+        <v>115.8123087915533</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[2010.9784897796935, 1640.0889742976017, 2273.3282190105674, 2289.5379632844306, 2205.8531333079436, 2208.003347354922, 2218.8435164245147]</t>
+          <t>[2231.779022874739, 2231.779022874739, 2231.779022874739, 2231.779022874739, 2231.779022874739, 2231.779022874739, 2231.779022874739]</t>
         </is>
       </c>
     </row>
@@ -654,17 +654,17 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>661.2951037669071</v>
+        <v>629.1804888206962</v>
       </c>
       <c r="D9" t="n">
-        <v>757.7170139704227</v>
+        <v>750.048724983121</v>
       </c>
       <c r="E9" t="n">
-        <v>76.27807605325179</v>
+        <v>28.77833844436665</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[3742.527507466394, 4196.078423844494, 4539.534791651236, 4098.317468325392, -224.80230462347572, 4234.629785171673, 3951.2698760829894]</t>
+          <t>[3742.527507466394, 4196.078423844494, 4539.5347916512355, 4098.317468325391, 0.0, 4234.629785171672, 3951.269876082989]</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[5923.124804577781, 6360.119366139865, 10833.395589589247, 9453.269519944151, 13288.902901987221, 4005.5982619466595, 20330.452225747737]</t>
+          <t>[5923.124804577783, 6360.1193661398665, 10833.395589589247, 9453.269519944153, 13288.902901987221, 4005.5982619466586, 20330.452225747737]</t>
         </is>
       </c>
     </row>
@@ -702,21 +702,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HW-add-add-a0.8-b0.4-g0.2</t>
+          <t>HW-add-add-a0.8-b0.2-g0.8</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>612.4359270238637</v>
+        <v>272.5526219361779</v>
       </c>
       <c r="D11" t="n">
-        <v>718.2815781071399</v>
+        <v>509.909574009765</v>
       </c>
       <c r="E11" t="n">
-        <v>66.8672170292096</v>
+        <v>73.23206748905014</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[3251.7748248909797, 1673.6035905415397, -111.42308291180143, 106.26011495988075, -487.0907394593212, 839.6207241846239, 817.2784122188984]</t>
+          <t>[1092.1316464467545, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0]</t>
         </is>
       </c>
     </row>
@@ -728,21 +728,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ARIMA(2,2,2)</t>
+          <t>(4, 0, 1)</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1507.754434637259</v>
+        <v>1539.836129722998</v>
       </c>
       <c r="D12" t="n">
-        <v>1721.486364771568</v>
+        <v>1748.041135970006</v>
       </c>
       <c r="E12" t="n">
-        <v>78.70756555438787</v>
+        <v>85.14373638978083</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[2554.636982368874, 3045.0023806846275, 3090.683550768701, 2989.2335535194484, 2967.263714763829, 2961.904674525177, 2943.0719512631845]</t>
+          <t>[2521.4965033909307, 3107.921648119547, 3434.6394051953857, 3314.5717584987005, 3204.401671238831, 3213.828698290291, 3242.163480433607]</t>
         </is>
       </c>
     </row>
@@ -764,11 +764,11 @@
         <v>1182.289171929961</v>
       </c>
       <c r="E13" t="n">
-        <v>34.35792362715212</v>
+        <v>34.35792362715211</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[3995.1375678260833, 4607.4318767095165, 3889.866697153984, 5076.7070167582415, 3866.022996406734, 4787.201123474417, 4240.699719131396]</t>
+          <t>[3995.137567826083, 4607.4318767095165, 3889.866697153984, 5076.7070167582415, 3866.022996406734, 4787.201123474417, 4240.699719131396]</t>
         </is>
       </c>
     </row>
@@ -780,21 +780,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ARIMA(0,1,2)</t>
+          <t>HW-None-add-a0.2-b0.2-g0.2</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3693.771571924263</v>
+        <v>4179.386435009455</v>
       </c>
       <c r="D14" t="n">
-        <v>4485.586812384538</v>
+        <v>4558.889805444956</v>
       </c>
       <c r="E14" t="n">
-        <v>105.4408089509267</v>
+        <v>110.2300068228071</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[6416.40100346984, 7319.266554669269, 7319.266554669269, 7319.266554669269, 7319.266554669269, 7319.266554669269, 7319.266554669269]</t>
+          <t>[9963.355936495373, 9093.249654844585, 12909.540397209335, 4701.932040376261, 6199.882153514304, 10294.283932551918, 10520.039760236428]</t>
         </is>
       </c>
     </row>
@@ -810,17 +810,17 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>813.8142576089285</v>
+        <v>813.8142576089267</v>
       </c>
       <c r="D15" t="n">
-        <v>1042.018799645556</v>
+        <v>1042.018799645555</v>
       </c>
       <c r="E15" t="n">
-        <v>47.05815960228255</v>
+        <v>47.05815960228237</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[1999.6856303250368, 2888.414753086127, 2285.4950040644817, 3438.3164577591397, 851.0645146672455, 3980.5226854842767, 7255.0756350169995]</t>
+          <t>[1999.6856303250358, 2888.4147530861255, 2285.4950040644794, 3438.316457759136, 851.0645146672414, 3980.522685484272, 7255.075635016992]</t>
         </is>
       </c>
     </row>
@@ -832,21 +832,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ARIMA(0,0,1)</t>
+          <t>HW-add-add-a0.4-b0.8-g0.4</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1337.3323657766</v>
+        <v>1174.134607135311</v>
       </c>
       <c r="D16" t="n">
-        <v>1656.692912786091</v>
+        <v>1414.69771922206</v>
       </c>
       <c r="E16" t="n">
-        <v>199.8524285938817</v>
+        <v>59.60133202210166</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[3355.678372876064, 2506.6183618493424, 2506.6183618493424, 2506.6183618493424, 2506.6183618493424, 2506.6183618493424, 2506.6183618493424]</t>
+          <t>[4146.010745904703, 1151.066959007348, 923.8347883342988, 0.0, 0.0, 1430.412786706728, 2932.06646731676]</t>
         </is>
       </c>
     </row>
@@ -862,17 +862,17 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>845.2735129622744</v>
+        <v>845.2735129622757</v>
       </c>
       <c r="D17" t="n">
-        <v>1138.349998467145</v>
+        <v>1138.349998467146</v>
       </c>
       <c r="E17" t="n">
-        <v>30.61848388345165</v>
+        <v>30.61848388345175</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[1778.769875224937, 5917.1944167942975, 3812.201810698857, 3841.6780998328663, 1371.1492304803573, 5222.494835632987, 5728.711105775819]</t>
+          <t>[1778.769875224938, 5917.1944167943, 3812.2018106988608, 3841.678099832871, 1371.1492304803633, 5222.494835632991, 5728.711105775824]</t>
         </is>
       </c>
     </row>
@@ -910,21 +910,21 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ARIMA(2,2,1)</t>
+          <t>HW-None-None-a0.4-b0.2-g0.2</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>390.7603210350317</v>
+        <v>557.604555707007</v>
       </c>
       <c r="D19" t="n">
-        <v>480.7282352667315</v>
+        <v>646.2399681060022</v>
       </c>
       <c r="E19" t="n">
-        <v>16.65475319213167</v>
+        <v>22.89194216784148</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[1977.7560602100361, 2182.374145238741, 2930.5545660112202, 2493.9617351063907, 2356.2924123814946, 2640.58972255431, 2584.58896725876]</t>
+          <t>[2403.2318899490488, 2403.2318899490488, 2403.2318899490488, 2403.2318899490488, 2403.2318899490488, 2403.2318899490488, 2403.2318899490488]</t>
         </is>
       </c>
     </row>
@@ -936,21 +936,21 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ARIMA(1,0,0)</t>
+          <t>(0, 1, 1)</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>238.7093013038641</v>
+        <v>500.4037626957896</v>
       </c>
       <c r="D20" t="n">
-        <v>295.1748895763454</v>
+        <v>585.1878684528102</v>
       </c>
       <c r="E20" t="n">
-        <v>15.10380222651205</v>
+        <v>35.18339173485032</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[1814.5750162899358, 1632.8061788200662, 1612.967452610048, 1610.8022021572508, 1610.5658810611428, 1610.540088358782, 1610.5372732758035]</t>
+          <t>[2140.5652677741055, 2140.5652677741055, 2140.5652677741055, 2140.5652677741055, 2140.5652677741055, 2140.5652677741055, 2140.5652677741055]</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[13309.390814341306, 15675.102730678838, 14702.795317026998, 18112.46747776542, 12228.802102781336, 18106.326375964993, 12800.412014436732]</t>
+          <t>[13309.390814341306, 15675.102730678838, 14702.795317026998, 18112.46747776542, 12228.802102781336, 18106.326375964993, 12800.412014436735]</t>
         </is>
       </c>
     </row>
@@ -1044,17 +1044,17 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>753.8750363185572</v>
+        <v>753.8750363185571</v>
       </c>
       <c r="D24" t="n">
-        <v>857.0794006714798</v>
+        <v>857.0794006714796</v>
       </c>
       <c r="E24" t="n">
-        <v>37.46481389812842</v>
+        <v>37.4648138981284</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[2527.3798932260815, 4513.587883384863, 3127.2099090136862, 2544.273556340064, 1728.7633328045927, 4501.291078256923, 2608.37842425509]</t>
+          <t>[2527.379893226081, 4513.587883384862, 3127.2099090136862, 2544.273556340064, 1728.763332804593, 4501.291078256923, 2608.37842425509]</t>
         </is>
       </c>
     </row>
@@ -1070,17 +1070,17 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1956.189867186835</v>
+        <v>1956.189867186844</v>
       </c>
       <c r="D25" t="n">
-        <v>2190.928740080053</v>
+        <v>2190.928740080059</v>
       </c>
       <c r="E25" t="n">
-        <v>34.71181413575682</v>
+        <v>34.71181413575703</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[4080.118614189629, 9145.00153834033, 12825.996529798138, 11036.7445640453, 6690.024764128787, 13880.517843664622, 9885.96398015094]</t>
+          <t>[4080.118614189635, 9145.001538340342, 12825.996529798167, 11036.744564045333, 6690.024764128804, 13880.517843664658, 9885.96398015097]</t>
         </is>
       </c>
     </row>
@@ -1092,21 +1092,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ARIMA(2,2,2)</t>
+          <t>HW-add-add-a0.4-b0.8-g0.4</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>942.6354311904785</v>
+        <v>733.682403504996</v>
       </c>
       <c r="D26" t="n">
-        <v>1098.979792610416</v>
+        <v>1161.708267609473</v>
       </c>
       <c r="E26" t="n">
-        <v>46.49548575664463</v>
+        <v>55.91017104030108</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[1486.7760908366213, 636.4746094460678, 703.2218219438887, 857.0201470973562, 832.5479273348462, 756.4094756217893, 708.4546967406427]</t>
+          <t>[1764.9262917443057, 169.0684976180042, 368.87775899727467, 0.0, 0.0, 0.0, 1374.6047230170411]</t>
         </is>
       </c>
     </row>
@@ -1125,14 +1125,14 @@
         <v>462.6527870165104</v>
       </c>
       <c r="D27" t="n">
-        <v>523.166464110311</v>
+        <v>523.1664641103107</v>
       </c>
       <c r="E27" t="n">
         <v>107.072613748397</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[1103.0104114234105, 547.126623282393, 532.8429018503169, 899.0081580557694, 178.3277506711936, 1030.6103517138818, 812.9085667212195]</t>
+          <t>[1103.0104114234105, 547.1266232823932, 532.842901850317, 899.0081580557696, 178.32775067119394, 1030.610351713882, 812.9085667212198]</t>
         </is>
       </c>
     </row>

</xml_diff>